<commit_message>
report update with new shell pacs added
</commit_message>
<xml_diff>
--- a/reports/pro-israel/pro-israel-F24-ie-report.xlsx
+++ b/reports/pro-israel/pro-israel-F24-ie-report.xlsx
@@ -121,12 +121,36 @@
     <x:t>07</x:t>
   </x:si>
   <x:si>
+    <x:t>C00863472</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EDW ACTION FUND</x:t>
+  </x:si>
+  <x:si>
     <x:t>H6IL09194</x:t>
   </x:si>
   <x:si>
     <x:t>FINE, LAURA</x:t>
   </x:si>
   <x:si>
+    <x:t>C00931774</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ARTICLE ONE PAC</x:t>
+  </x:si>
+  <x:si>
+    <x:t>H2NC06114</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FOUSHEE, VALERIE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>04</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NC</x:t>
+  </x:si>
+  <x:si>
     <x:t>H6IL07339</x:t>
   </x:si>
   <x:si>
@@ -157,19 +181,19 @@
     <x:t>02</x:t>
   </x:si>
   <x:si>
+    <x:t>H6NJ11310</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WAY, TAHESHA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11</x:t>
+  </x:si>
+  <x:si>
     <x:t>C00710848</x:t>
   </x:si>
   <x:si>
     <x:t>DMFI PAC</x:t>
-  </x:si>
-  <x:si>
-    <x:t>H6NJ11310</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WAY, TAHESHA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -240,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J12" totalsRowShown="0">
-  <x:autoFilter ref="A1:J12"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:J15" totalsRowShown="0">
+  <x:autoFilter ref="A1:J15"/>
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="committee_id" dataDxfId="0"/>
     <x:tableColumn id="2" name="committee_name" dataDxfId="0"/>
@@ -546,7 +570,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:J12"/>
+  <x:dimension ref="A1:J15"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="11" max="16384" width="9.140625" style="1" customWidth="1"/>
@@ -788,16 +812,16 @@
     </x:row>
     <x:row r="8" spans="1:10">
       <x:c r="A8" s="1" t="s">
-        <x:v>21</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B8" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C8" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D8" s="1" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E8" s="1" t="s">
         <x:v>14</x:v>
@@ -809,7 +833,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="H8" s="1">
-        <x:v>4383749</x:v>
+        <x:v>500346</x:v>
       </x:c>
       <x:c r="I8" s="1">
         <x:v>2026</x:v>
@@ -820,10 +844,10 @@
     </x:row>
     <x:row r="9" spans="1:10">
       <x:c r="A9" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C9" s="1" t="s">
         <x:v>37</x:v>
@@ -835,114 +859,210 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="F9" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G9" s="1" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="H9" s="1">
-        <x:v>59748</x:v>
+        <x:v>4383749</x:v>
       </x:c>
       <x:c r="I9" s="1">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="J9" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:10">
       <x:c r="A10" s="1" t="s">
-        <x:v>30</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B10" s="1" t="s">
-        <x:v>31</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="C10" s="1" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="D10" s="1" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="E10" s="1" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F10" s="1" t="s">
-        <x:v>34</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="G10" s="1" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="H10" s="1">
-        <x:v>2326917</x:v>
+        <x:v>600000</x:v>
       </x:c>
       <x:c r="I10" s="1">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="J10" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:10">
       <x:c r="A11" s="1" t="s">
-        <x:v>42</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B11" s="1" t="s">
-        <x:v>43</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C11" s="1" t="s">
-        <x:v>44</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D11" s="1" t="s">
-        <x:v>45</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E11" s="1" t="s">
         <x:v>14</x:v>
       </x:c>
       <x:c r="F11" s="1" t="s">
-        <x:v>46</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="G11" s="1" t="s">
         <x:v>16</x:v>
       </x:c>
       <x:c r="H11" s="1">
-        <x:v>4379246</x:v>
+        <x:v>59748</x:v>
       </x:c>
       <x:c r="I11" s="1">
         <x:v>2026</x:v>
       </x:c>
       <x:c r="J11" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:10">
       <x:c r="A12" s="1" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B12" s="1" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C12" s="1" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="B12" s="1" t="s">
+      <x:c r="D12" s="1" t="s">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="C12" s="1" t="s">
+      <x:c r="E12" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F12" s="1" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G12" s="1" t="s">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="D12" s="1" t="s">
+      <x:c r="H12" s="1">
+        <x:v>2326917</x:v>
+      </x:c>
+      <x:c r="I12" s="1">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="J12" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:10">
+      <x:c r="A13" s="1" t="s">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E12" s="1" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F12" s="1" t="s">
+      <x:c r="B13" s="1" t="s">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="G12" s="1" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="H12" s="1">
+      <x:c r="C13" s="1" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D13" s="1" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="G13" s="1" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="H13" s="1">
+        <x:v>4379246</x:v>
+      </x:c>
+      <x:c r="I13" s="1">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="J13" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:10">
+      <x:c r="A14" s="1" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B14" s="1" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C14" s="1" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D14" s="1" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F14" s="1" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G14" s="1" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="H14" s="1">
+        <x:v>350000</x:v>
+      </x:c>
+      <x:c r="I14" s="1">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="J14" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:10">
+      <x:c r="A15" s="1" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B15" s="1" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C15" s="1" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D15" s="1" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E15" s="1" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F15" s="1" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G15" s="1" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="H15" s="1">
         <x:v>38952</x:v>
       </x:c>
-      <x:c r="I12" s="1">
-        <x:v>2026</x:v>
-      </x:c>
-      <x:c r="J12" s="1" t="s">
+      <x:c r="I15" s="1">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="J15" s="1" t="s">
         <x:v>25</x:v>
       </x:c>
     </x:row>

</xml_diff>